<commit_message>
added working age population analysis, added top1 incclass analysis, changed jointplots to represent population size
</commit_message>
<xml_diff>
--- a/data_input/density_class_combo_emissions.xlsx
+++ b/data_input/density_class_combo_emissions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>tenure_lab</t>
+          <t>inc_lab</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -473,23 +473,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5885.438713979452</v>
+        <v>5239.881575399763</v>
       </c>
       <c r="D2" t="n">
-        <v>3815.326299624254</v>
+        <v>3606.039305736101</v>
       </c>
       <c r="E2" t="n">
-        <v>4356.990681273705</v>
+        <v>4027.631540995803</v>
       </c>
       <c r="F2" t="n">
-        <v>4603.686594037779</v>
+        <v>4225.295990781868</v>
       </c>
       <c r="G2" t="n">
-        <v>2254475</v>
+        <v>1460025</v>
       </c>
     </row>
     <row r="3">
@@ -500,23 +500,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>priate rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7022.35421696803</v>
+        <v>6296.499469910782</v>
       </c>
       <c r="D3" t="n">
-        <v>3630.09418701205</v>
+        <v>4606.05448554169</v>
       </c>
       <c r="E3" t="n">
-        <v>4945.394340895863</v>
+        <v>4945.966629610308</v>
       </c>
       <c r="F3" t="n">
-        <v>5135.809271442951</v>
+        <v>5198.621803668272</v>
       </c>
       <c r="G3" t="n">
-        <v>183240</v>
+        <v>321830</v>
       </c>
     </row>
     <row r="4">
@@ -527,50 +527,50 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4798.163975956058</v>
+        <v>4147.878472864532</v>
       </c>
       <c r="D4" t="n">
-        <v>2755.057301259241</v>
+        <v>2930.664823023083</v>
       </c>
       <c r="E4" t="n">
-        <v>3587.449069498815</v>
+        <v>3708.697259251159</v>
       </c>
       <c r="F4" t="n">
-        <v>3682.029854053232</v>
+        <v>3623.984453597483</v>
       </c>
       <c r="G4" t="n">
-        <v>629555</v>
+        <v>1254925</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>low suburban</t>
+          <t>high suburban</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6856.560316007463</v>
+        <v>7839.256496930972</v>
       </c>
       <c r="D5" t="n">
-        <v>4517.508062458724</v>
+        <v>5818.351726334409</v>
       </c>
       <c r="E5" t="n">
-        <v>4979.940841848915</v>
+        <v>6274.560713722933</v>
       </c>
       <c r="F5" t="n">
-        <v>5333.487515541005</v>
+        <v>6551.682412677812</v>
       </c>
       <c r="G5" t="n">
-        <v>2077660</v>
+        <v>31610</v>
       </c>
     </row>
     <row r="6">
@@ -581,23 +581,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>priate rental</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6875.952690843332</v>
+        <v>6478.397137832225</v>
       </c>
       <c r="D6" t="n">
-        <v>3891.541550423678</v>
+        <v>4515.5740240542</v>
       </c>
       <c r="E6" t="n">
-        <v>5633.779993692066</v>
+        <v>4791.567699257903</v>
       </c>
       <c r="F6" t="n">
-        <v>5508.763557162785</v>
+        <v>5144.276640100557</v>
       </c>
       <c r="G6" t="n">
-        <v>135380</v>
+        <v>1300790</v>
       </c>
     </row>
     <row r="7">
@@ -608,77 +608,77 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5490.845356833731</v>
+        <v>6985.978957389824</v>
       </c>
       <c r="D7" t="n">
-        <v>3441.688371424738</v>
+        <v>5145.39500620411</v>
       </c>
       <c r="E7" t="n">
-        <v>4502.323700768236</v>
+        <v>5446.707908948989</v>
       </c>
       <c r="F7" t="n">
-        <v>4484.295282448736</v>
+        <v>5756.197445372978</v>
       </c>
       <c r="G7" t="n">
-        <v>442365</v>
+        <v>299315</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rural</t>
+          <t>low suburban</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5811.008847314267</v>
+        <v>4975.821285061419</v>
       </c>
       <c r="D8" t="n">
-        <v>4854.986454913957</v>
+        <v>3402.441236111623</v>
       </c>
       <c r="E8" t="n">
-        <v>5233.68324629469</v>
+        <v>4106.182121580295</v>
       </c>
       <c r="F8" t="n">
-        <v>5283.3404487044</v>
+        <v>4147.656691083408</v>
       </c>
       <c r="G8" t="n">
-        <v>2156355</v>
+        <v>1022635</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rural</t>
+          <t>low suburban</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>priate rental</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6706.930190072303</v>
+        <v>5891.795033361172</v>
       </c>
       <c r="D9" t="n">
-        <v>4579.438194532134</v>
+        <v>4849.432684221696</v>
       </c>
       <c r="E9" t="n">
-        <v>5996.25455248341</v>
+        <v>5136.783923530994</v>
       </c>
       <c r="F9" t="n">
-        <v>5819.719372392814</v>
+        <v>5253.698891161213</v>
       </c>
       <c r="G9" t="n">
-        <v>155555</v>
+        <v>33240</v>
       </c>
     </row>
     <row r="10">
@@ -689,185 +689,320 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5991.233202686336</v>
+        <v>5012.11485654138</v>
       </c>
       <c r="D10" t="n">
-        <v>3860.128216891741</v>
+        <v>4483.367434927012</v>
       </c>
       <c r="E10" t="n">
-        <v>5078.548332588484</v>
+        <v>4638.513400104408</v>
       </c>
       <c r="F10" t="n">
-        <v>5002.114521188762</v>
+        <v>4693.127272919302</v>
       </c>
       <c r="G10" t="n">
-        <v>248880</v>
+        <v>1252035</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5585.02341419302</v>
+        <v>5954.567676114597</v>
       </c>
       <c r="D11" t="n">
-        <v>3642.814579523156</v>
+        <v>5752.025447409799</v>
       </c>
       <c r="E11" t="n">
-        <v>4326.264742248695</v>
+        <v>5827.566164099035</v>
       </c>
       <c r="F11" t="n">
-        <v>4470.091869553392</v>
+        <v>5840.431362930617</v>
       </c>
       <c r="G11" t="n">
-        <v>2688645</v>
+        <v>338570</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>priate rental</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8208.365989629841</v>
+        <v>5596.44071680236</v>
       </c>
       <c r="D12" t="n">
-        <v>4116.620398576352</v>
+        <v>4154.099087841259</v>
       </c>
       <c r="E12" t="n">
-        <v>5263.093465643761</v>
+        <v>4732.341014569944</v>
       </c>
       <c r="F12" t="n">
-        <v>5712.79332987343</v>
+        <v>4803.805458445877</v>
       </c>
       <c r="G12" t="n">
-        <v>333340</v>
+        <v>931530</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5929.426064892786</v>
+        <v>6025.837878424099</v>
       </c>
       <c r="D13" t="n">
-        <v>2555.855974029972</v>
+        <v>5725.861715738954</v>
       </c>
       <c r="E13" t="n">
-        <v>3243.709742277852</v>
+        <v>5888.829784664998</v>
       </c>
       <c r="F13" t="n">
-        <v>3743.175380869615</v>
+        <v>5882.339790873262</v>
       </c>
       <c r="G13" t="n">
-        <v>1154980</v>
+        <v>39515</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>very urban</t>
+          <t>urban</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4468.895865610992</v>
+        <v>4991.343539869354</v>
       </c>
       <c r="D14" t="n">
-        <v>3334.619606783634</v>
+        <v>3440.4850817275</v>
       </c>
       <c r="E14" t="n">
-        <v>4051.884041148074</v>
+        <v>4022.01160596818</v>
       </c>
       <c r="F14" t="n">
-        <v>3976.820888672693</v>
+        <v>4118.962958383304</v>
       </c>
       <c r="G14" t="n">
-        <v>1732915</v>
+        <v>1834780</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>very urban</t>
+          <t>urban</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>priate rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9377.689862340778</v>
+        <v>6007.608793897572</v>
       </c>
       <c r="D15" t="n">
-        <v>4237.505181626087</v>
+        <v>4334.682567468236</v>
       </c>
       <c r="E15" t="n">
-        <v>4699.19515688581</v>
+        <v>4850.112221345489</v>
       </c>
       <c r="F15" t="n">
-        <v>5753.396339434621</v>
+        <v>5010.628951014196</v>
       </c>
       <c r="G15" t="n">
-        <v>684640</v>
+        <v>400205</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>urban</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>poorest 50%</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3964.217565699944</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2672.676401078681</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3350.080688988018</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3334.263836188665</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1905790</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>urban</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>top 1%</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>10641.42374291252</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8124.520216181863</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8603.13973200349</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8993.055855775339</v>
+      </c>
+      <c r="G17" t="n">
+        <v>37940</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>very urban</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>social rental</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>6263.467842375323</v>
-      </c>
-      <c r="D16" t="n">
-        <v>2396.895055655953</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2859.941984478597</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3595.061716747118</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1361870</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>51-90%</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3742.633389894152</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2848.904155705424</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3391.898215711025</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3343.833494255407</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1418650</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>91-99%</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4618.428265112355</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3616.504143300569</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4208.725913126018</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4163.09605866624</v>
+      </c>
+      <c r="G19" t="n">
+        <v>392465</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>poorest 50%</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3730.869870779442</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2455.158334517435</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2852.937627357822</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2972.97586500313</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1925210</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>top 1%</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7396.817729346041</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6489.808354723963</v>
+      </c>
+      <c r="E21" t="n">
+        <v>7069.494470871497</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7006.40375645325</v>
+      </c>
+      <c r="G21" t="n">
+        <v>46530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrected missing values of mobility for 0.04% population
</commit_message>
<xml_diff>
--- a/data_input/density_class_combo_emissions.xlsx
+++ b/data_input/density_class_combo_emissions.xlsx
@@ -477,16 +477,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5885.438713979452</v>
+        <v>4911.496665397945</v>
       </c>
       <c r="D2" t="n">
-        <v>3815.326299624254</v>
+        <v>3832.388957812942</v>
       </c>
       <c r="E2" t="n">
-        <v>4356.990681273705</v>
+        <v>4460.868559661682</v>
       </c>
       <c r="F2" t="n">
-        <v>4603.686594037779</v>
+        <v>4416.405685633563</v>
       </c>
       <c r="G2" t="n">
         <v>2254475</v>
@@ -504,16 +504,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7022.35421696803</v>
+        <v>7091.124522305787</v>
       </c>
       <c r="D3" t="n">
-        <v>3630.09418701205</v>
+        <v>3994.548276334268</v>
       </c>
       <c r="E3" t="n">
-        <v>4945.394340895863</v>
+        <v>4890.021147650991</v>
       </c>
       <c r="F3" t="n">
-        <v>5135.809271442951</v>
+        <v>5216.428773485509</v>
       </c>
       <c r="G3" t="n">
         <v>183240</v>
@@ -531,16 +531,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4798.163975956058</v>
+        <v>4733.062415568348</v>
       </c>
       <c r="D4" t="n">
-        <v>2755.057301259241</v>
+        <v>2943.381864269975</v>
       </c>
       <c r="E4" t="n">
-        <v>3587.449069498815</v>
+        <v>3482.771214268875</v>
       </c>
       <c r="F4" t="n">
-        <v>3682.029854053232</v>
+        <v>3660.496677094018</v>
       </c>
       <c r="G4" t="n">
         <v>629555</v>
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6856.560316007463</v>
+        <v>5740.136885743651</v>
       </c>
       <c r="D5" t="n">
-        <v>4517.508062458724</v>
+        <v>4464.679503023975</v>
       </c>
       <c r="E5" t="n">
-        <v>4979.940841848915</v>
+        <v>5072.864022052945</v>
       </c>
       <c r="F5" t="n">
-        <v>5333.487515541005</v>
+        <v>5087.636108218379</v>
       </c>
       <c r="G5" t="n">
         <v>2077660</v>
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6875.952690843332</v>
+        <v>7079.880374933086</v>
       </c>
       <c r="D6" t="n">
-        <v>3891.541550423678</v>
+        <v>4296.286589718811</v>
       </c>
       <c r="E6" t="n">
-        <v>5633.779993692066</v>
+        <v>5464.781080939631</v>
       </c>
       <c r="F6" t="n">
-        <v>5508.763557162785</v>
+        <v>5576.43228163279</v>
       </c>
       <c r="G6" t="n">
         <v>135380</v>
@@ -612,16 +612,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5490.845356833731</v>
+        <v>5298.232799341185</v>
       </c>
       <c r="D7" t="n">
-        <v>3441.688371424738</v>
+        <v>3671.8256170858</v>
       </c>
       <c r="E7" t="n">
-        <v>4502.323700768236</v>
+        <v>4387.737022256679</v>
       </c>
       <c r="F7" t="n">
-        <v>4484.295282448736</v>
+        <v>4436.383115235086</v>
       </c>
       <c r="G7" t="n">
         <v>442365</v>
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5811.008847314267</v>
+        <v>5581.095721343929</v>
       </c>
       <c r="D8" t="n">
-        <v>4854.986454913957</v>
+        <v>4636.536377987034</v>
       </c>
       <c r="E8" t="n">
-        <v>5233.68324629469</v>
+        <v>5182.763905534606</v>
       </c>
       <c r="F8" t="n">
-        <v>5283.3404487044</v>
+        <v>5145.789977600044</v>
       </c>
       <c r="G8" t="n">
         <v>2156355</v>
@@ -666,16 +666,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6706.930190072303</v>
+        <v>6958.997753521457</v>
       </c>
       <c r="D9" t="n">
-        <v>4579.438194532134</v>
+        <v>4768.246960130776</v>
       </c>
       <c r="E9" t="n">
-        <v>5996.25455248341</v>
+        <v>5891.500796786215</v>
       </c>
       <c r="F9" t="n">
-        <v>5819.719372392814</v>
+        <v>5877.561576806165</v>
       </c>
       <c r="G9" t="n">
         <v>155555</v>
@@ -693,16 +693,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5991.233202686336</v>
+        <v>5994.614475497911</v>
       </c>
       <c r="D10" t="n">
-        <v>3860.128216891741</v>
+        <v>3985.362503925388</v>
       </c>
       <c r="E10" t="n">
-        <v>5078.548332588484</v>
+        <v>4739.562862882447</v>
       </c>
       <c r="F10" t="n">
-        <v>5002.114521188762</v>
+        <v>4864.775676297048</v>
       </c>
       <c r="G10" t="n">
         <v>248880</v>
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5585.02341419302</v>
+        <v>4825.426378082513</v>
       </c>
       <c r="D11" t="n">
-        <v>3642.814579523156</v>
+        <v>3728.5491915398</v>
       </c>
       <c r="E11" t="n">
-        <v>4326.264742248695</v>
+        <v>4418.212094654136</v>
       </c>
       <c r="F11" t="n">
-        <v>4470.091869553392</v>
+        <v>4347.599939732647</v>
       </c>
       <c r="G11" t="n">
         <v>2688645</v>
@@ -747,16 +747,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8208.365989629841</v>
+        <v>8088.606815906125</v>
       </c>
       <c r="D12" t="n">
-        <v>4116.620398576352</v>
+        <v>4545.78052843883</v>
       </c>
       <c r="E12" t="n">
-        <v>5263.093465643761</v>
+        <v>5306.234450741997</v>
       </c>
       <c r="F12" t="n">
-        <v>5712.79332987343</v>
+        <v>5811.714061457236</v>
       </c>
       <c r="G12" t="n">
         <v>333340</v>
@@ -774,16 +774,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5929.426064892786</v>
+        <v>5589.101621420755</v>
       </c>
       <c r="D13" t="n">
-        <v>2555.855974029972</v>
+        <v>2772.082560444347</v>
       </c>
       <c r="E13" t="n">
-        <v>3243.709742277852</v>
+        <v>3229.65668305242</v>
       </c>
       <c r="F13" t="n">
-        <v>3743.175380869615</v>
+        <v>3705.124386992486</v>
       </c>
       <c r="G13" t="n">
         <v>1154980</v>
@@ -801,16 +801,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4468.895865610992</v>
+        <v>4694.689418447797</v>
       </c>
       <c r="D14" t="n">
-        <v>3334.619606783634</v>
+        <v>3537.607176466083</v>
       </c>
       <c r="E14" t="n">
-        <v>4051.884041148074</v>
+        <v>4012.144686159684</v>
       </c>
       <c r="F14" t="n">
-        <v>3976.820888672693</v>
+        <v>4064.146491808312</v>
       </c>
       <c r="G14" t="n">
         <v>1732915</v>
@@ -828,16 +828,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9377.689862340778</v>
+        <v>9016.349284731297</v>
       </c>
       <c r="D15" t="n">
-        <v>4237.505181626087</v>
+        <v>4226.140667004545</v>
       </c>
       <c r="E15" t="n">
-        <v>4699.19515688581</v>
+        <v>4794.068730447932</v>
       </c>
       <c r="F15" t="n">
-        <v>5753.396339434621</v>
+        <v>5707.656853157927</v>
       </c>
       <c r="G15" t="n">
         <v>684640</v>
@@ -855,16 +855,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6263.467842375323</v>
+        <v>6169.284248133609</v>
       </c>
       <c r="D16" t="n">
-        <v>2396.895055655953</v>
+        <v>2605.059751634401</v>
       </c>
       <c r="E16" t="n">
-        <v>2859.941984478597</v>
+        <v>2924.00567414758</v>
       </c>
       <c r="F16" t="n">
-        <v>3595.061716747118</v>
+        <v>3655.588837015792</v>
       </c>
       <c r="G16" t="n">
         <v>1361870</v>

</xml_diff>

<commit_message>
ran all analysis again with imputed mobility values
</commit_message>
<xml_diff>
--- a/data_input/density_class_combo_emissions.xlsx
+++ b/data_input/density_class_combo_emissions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>tenure_lab</t>
+          <t>inc_lab</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -473,23 +473,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4911.496665397945</v>
+        <v>4453.144266790459</v>
       </c>
       <c r="D2" t="n">
-        <v>3832.388957812942</v>
+        <v>3646.431619576658</v>
       </c>
       <c r="E2" t="n">
-        <v>4460.868559661682</v>
+        <v>4115.614891975494</v>
       </c>
       <c r="F2" t="n">
-        <v>4416.405685633563</v>
+        <v>4082.701417579527</v>
       </c>
       <c r="G2" t="n">
-        <v>2254475</v>
+        <v>1460025</v>
       </c>
     </row>
     <row r="3">
@@ -500,23 +500,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>private rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7091.124522305787</v>
+        <v>5329.527485225737</v>
       </c>
       <c r="D3" t="n">
-        <v>3994.548276334268</v>
+        <v>4613.654804490987</v>
       </c>
       <c r="E3" t="n">
-        <v>4890.021147650991</v>
+        <v>5016.472643173143</v>
       </c>
       <c r="F3" t="n">
-        <v>5216.428773485509</v>
+        <v>4994.031894015753</v>
       </c>
       <c r="G3" t="n">
-        <v>183240</v>
+        <v>321830</v>
       </c>
     </row>
     <row r="4">
@@ -527,50 +527,50 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4733.062415568348</v>
+        <v>4310.389520408152</v>
       </c>
       <c r="D4" t="n">
-        <v>2943.381864269975</v>
+        <v>3030.934174804303</v>
       </c>
       <c r="E4" t="n">
-        <v>3482.771214268875</v>
+        <v>3597.287586063643</v>
       </c>
       <c r="F4" t="n">
-        <v>3660.496677094018</v>
+        <v>3633.974716834935</v>
       </c>
       <c r="G4" t="n">
-        <v>629555</v>
+        <v>1254925</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>low suburban</t>
+          <t>high suburban</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5740.136885743651</v>
+        <v>6720.365585093559</v>
       </c>
       <c r="D5" t="n">
-        <v>4464.679503023975</v>
+        <v>5640.888183672378</v>
       </c>
       <c r="E5" t="n">
-        <v>5072.864022052945</v>
+        <v>6251.912747171431</v>
       </c>
       <c r="F5" t="n">
-        <v>5087.636108218379</v>
+        <v>6216.2698157772</v>
       </c>
       <c r="G5" t="n">
-        <v>2077660</v>
+        <v>31610</v>
       </c>
     </row>
     <row r="6">
@@ -581,23 +581,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>private rental</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7079.880374933086</v>
+        <v>5467.86178759557</v>
       </c>
       <c r="D6" t="n">
-        <v>4296.286589718811</v>
+        <v>4486.194038712213</v>
       </c>
       <c r="E6" t="n">
-        <v>5464.781080939631</v>
+        <v>4886.520804853755</v>
       </c>
       <c r="F6" t="n">
-        <v>5576.43228163279</v>
+        <v>4931.774359003823</v>
       </c>
       <c r="G6" t="n">
-        <v>135380</v>
+        <v>1300790</v>
       </c>
     </row>
     <row r="7">
@@ -608,77 +608,77 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5298.232799341185</v>
+        <v>6000.931866518476</v>
       </c>
       <c r="D7" t="n">
-        <v>3671.8256170858</v>
+        <v>5072.593238091414</v>
       </c>
       <c r="E7" t="n">
-        <v>4387.737022256679</v>
+        <v>5502.938458333406</v>
       </c>
       <c r="F7" t="n">
-        <v>4436.383115235086</v>
+        <v>5519.850505319175</v>
       </c>
       <c r="G7" t="n">
-        <v>442365</v>
+        <v>299315</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rural</t>
+          <t>low suburban</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5581.095721343929</v>
+        <v>4685.663852350664</v>
       </c>
       <c r="D8" t="n">
-        <v>4636.536377987034</v>
+        <v>3455.406319909788</v>
       </c>
       <c r="E8" t="n">
-        <v>5182.763905534606</v>
+        <v>4128.775579663262</v>
       </c>
       <c r="F8" t="n">
-        <v>5145.789977600044</v>
+        <v>4099.655332896744</v>
       </c>
       <c r="G8" t="n">
-        <v>2156355</v>
+        <v>1022635</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rural</t>
+          <t>low suburban</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>private rental</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6958.997753521457</v>
+        <v>5962.187195453771</v>
       </c>
       <c r="D9" t="n">
-        <v>4768.246960130776</v>
+        <v>5061.975387101282</v>
       </c>
       <c r="E9" t="n">
-        <v>5891.500796786215</v>
+        <v>5525.929044072946</v>
       </c>
       <c r="F9" t="n">
-        <v>5877.561576806165</v>
+        <v>5519.005167675236</v>
       </c>
       <c r="G9" t="n">
-        <v>155555</v>
+        <v>33240</v>
       </c>
     </row>
     <row r="10">
@@ -689,185 +689,320 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5994.614475497911</v>
+        <v>4873.18152700621</v>
       </c>
       <c r="D10" t="n">
-        <v>3985.362503925388</v>
+        <v>4279.98135622386</v>
       </c>
       <c r="E10" t="n">
-        <v>4739.562862882447</v>
+        <v>4597.352975827813</v>
       </c>
       <c r="F10" t="n">
-        <v>4864.775676297048</v>
+        <v>4586.967208721424</v>
       </c>
       <c r="G10" t="n">
-        <v>248880</v>
+        <v>1252035</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4825.426378082513</v>
+        <v>6014.747791854893</v>
       </c>
       <c r="D11" t="n">
-        <v>3728.5491915398</v>
+        <v>5466.760807091032</v>
       </c>
       <c r="E11" t="n">
-        <v>4418.212094654136</v>
+        <v>5687.72771419366</v>
       </c>
       <c r="F11" t="n">
-        <v>4347.599939732647</v>
+        <v>5714.241006833312</v>
       </c>
       <c r="G11" t="n">
-        <v>2688645</v>
+        <v>338570</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>private rental</t>
+          <t>poorest 50%</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8088.606815906125</v>
+        <v>5212.468664148926</v>
       </c>
       <c r="D12" t="n">
-        <v>4545.78052843883</v>
+        <v>4024.679710318929</v>
       </c>
       <c r="E12" t="n">
-        <v>5306.234450741997</v>
+        <v>4710.040300729996</v>
       </c>
       <c r="F12" t="n">
-        <v>5811.714061457236</v>
+        <v>4664.307243981962</v>
       </c>
       <c r="G12" t="n">
-        <v>333340</v>
+        <v>931530</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>urban</t>
+          <t>rural</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>social rental</t>
+          <t>top 1%</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5589.101621420755</v>
+        <v>6231.775414810246</v>
       </c>
       <c r="D13" t="n">
-        <v>2772.082560444347</v>
+        <v>5317.831319386308</v>
       </c>
       <c r="E13" t="n">
-        <v>3229.65668305242</v>
+        <v>5749.50764497883</v>
       </c>
       <c r="F13" t="n">
-        <v>3705.124386992486</v>
+        <v>5762.155506038554</v>
       </c>
       <c r="G13" t="n">
-        <v>1154980</v>
+        <v>39515</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>very urban</t>
+          <t>urban</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>owner occupied</t>
+          <t>51-90%</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4694.689418447797</v>
+        <v>4435.780155409547</v>
       </c>
       <c r="D14" t="n">
-        <v>3537.607176466083</v>
+        <v>3552.642230397776</v>
       </c>
       <c r="E14" t="n">
-        <v>4012.144686159684</v>
+        <v>4096.373602690445</v>
       </c>
       <c r="F14" t="n">
-        <v>4064.146491808312</v>
+        <v>4045.292397797053</v>
       </c>
       <c r="G14" t="n">
-        <v>1732915</v>
+        <v>1834780</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>very urban</t>
+          <t>urban</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>private rental</t>
+          <t>91-99%</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9016.349284731297</v>
+        <v>5157.330774527875</v>
       </c>
       <c r="D15" t="n">
-        <v>4226.140667004545</v>
+        <v>4417.269085192635</v>
       </c>
       <c r="E15" t="n">
-        <v>4794.068730447932</v>
+        <v>4931.809868811791</v>
       </c>
       <c r="F15" t="n">
-        <v>5707.656853157927</v>
+        <v>4859.554899336023</v>
       </c>
       <c r="G15" t="n">
-        <v>684640</v>
+        <v>400205</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>urban</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>poorest 50%</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4202.389612773768</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2817.369555930721</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3300.284776044617</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3405.082180198431</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1905790</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>urban</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>top 1%</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9306.47532605302</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8145.191972325329</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8545.517828344866</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8635.67573876702</v>
+      </c>
+      <c r="G17" t="n">
+        <v>37940</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>very urban</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>social rental</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>6169.284248133609</v>
-      </c>
-      <c r="D16" t="n">
-        <v>2605.059751634401</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2924.00567414758</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3655.588837015792</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1361870</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>51-90%</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3940.657793975894</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3028.003469168721</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3394.623494181177</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3439.477062876742</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1418650</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>91-99%</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4884.409403338443</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3821.926375146114</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4201.973637091087</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4277.570763166683</v>
+      </c>
+      <c r="G19" t="n">
+        <v>392465</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>poorest 50%</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3927.744151723606</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2596.928732785874</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2895.308286387439</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3078.822364321089</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1925210</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>very urban</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>top 1%</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8053.363818392081</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6556.834847650395</v>
+      </c>
+      <c r="E21" t="n">
+        <v>7243.269085600765</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7274.184209311002</v>
+      </c>
+      <c r="G21" t="n">
+        <v>46530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>